<commit_message>
Added YAML loading support in Tab2 for DRM-restricted environment
</commit_message>
<xml_diff>
--- a/plans/default_mission_plan.xlsx
+++ b/plans/default_mission_plan.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,41 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002A2A2A"/>
-        <bgColor rgb="002A2A2A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F9FF"/>
-        <bgColor rgb="00F2F9FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFBF0"/>
-        <bgColor rgb="00FFFBF0"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -74,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,200 +413,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Satellite</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Activity Sequence ID</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Pre Activity Sequence ID</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>최소 pass contact 시간</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>X-Band 여부</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>NEONSAT1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>TC_히터_온</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>101</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>NEONSAT1</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>TM_덤프_X밴드</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>102</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>101</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>SPACEEYE-T1</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>안테나_전개</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>201</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>SPACEEYE-T1</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>배터리_초기화</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>202</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>201</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Sat_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Min_El</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Required_Cap</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Min_Duration</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Pre_Req_Main</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Sequence_ID</t>
         </is>
       </c>
     </row>

</xml_diff>